<commit_message>
Adding forecast coverage image
including formatting corrections to the original Excel dataset.
</commit_message>
<xml_diff>
--- a/datasets/pipeline_forecast_attainments.xlsx
+++ b/datasets/pipeline_forecast_attainments.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Anil\GitHub\newbridge-saas-operating-system\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE68081-CAFF-438C-B16B-FAE3A866ACD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4923A09B-8367-4CFF-92C9-38A62A1F474A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1950" yWindow="0" windowWidth="20370" windowHeight="15480" xr2:uid="{76865BDF-23CF-4B29-B294-8B6645415571}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Forecast Coverage" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -96,11 +96,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
+    <numFmt numFmtId="167" formatCode="#.00,,&quot;M&quot;;[Red]#.00,,&quot;M&quot;"/>
+    <numFmt numFmtId="168" formatCode="#0.00,,&quot;M&quot;;[Red]#.00,,&quot;M&quot;"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="8"/>
       <color theme="1"/>
@@ -114,8 +115,14 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
-      <sz val="8"/>
+      <sz val="9"/>
       <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
@@ -129,7 +136,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -137,21 +144,98 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -487,308 +571,311 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4319F192-A262-4AC2-A2B9-A5F22F786F0E}">
-  <dimension ref="B2:H14"/>
+  <dimension ref="B1:H15"/>
   <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="2" max="2" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="C2" s="4" t="s">
+    <row r="1" spans="2:8" ht="11.25" thickBot="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:8" ht="12" x14ac:dyDescent="0.2">
+      <c r="B2" s="1"/>
+      <c r="C2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4" t="s">
+      <c r="D2" s="3"/>
+      <c r="E2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4" t="s">
+      <c r="F2" s="3"/>
+      <c r="G2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="4"/>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="B3" s="2" t="s">
+      <c r="H2" s="3"/>
+    </row>
+    <row r="3" spans="2:8" ht="12" x14ac:dyDescent="0.2">
+      <c r="B3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="B4" t="s">
+    <row r="4" spans="2:8" ht="12" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="10">
         <v>2145843.0924399644</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="5">
         <v>1.0516723050613055</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="10">
         <v>-5316462.195008792</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="5">
         <v>0.87197859090665175</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="10">
         <v>-13767627.59341744</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="5">
         <v>0.66847293938505126</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="B5" t="s">
+    <row r="5" spans="2:8" ht="12" x14ac:dyDescent="0.2">
+      <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="10">
         <v>3376856.5422686934</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="5">
         <v>1.0976239298318851</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="10">
         <v>-3263444.7762306258</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="5">
         <v>0.90565477098090474</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="10">
         <v>-11044067.856143363</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="5">
         <v>0.68071924526519401</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="B6" t="s">
+    <row r="6" spans="2:8" ht="12" x14ac:dyDescent="0.2">
+      <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="10">
         <v>412410.56413429603</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="5">
         <v>1.0161668420891736</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="10">
         <v>-1265414.7946229205</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="5">
         <v>0.95039467234570907</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="10">
         <v>-3160555.4089337587</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="5">
         <v>0.87610356122284838</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="B7" t="s">
+    <row r="7" spans="2:8" ht="12" x14ac:dyDescent="0.2">
+      <c r="B7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="10">
         <v>450519.63611060753</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="5">
         <v>1.025874295465063</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="10">
         <v>-616374.07395501062</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="5">
         <v>0.9646003334189831</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="10">
         <v>-1615517.5884540528</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="5">
         <v>0.90721740838305265</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="B8" t="s">
+    <row r="8" spans="2:8" ht="12" x14ac:dyDescent="0.2">
+      <c r="B8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="10">
         <v>398654.47068489343</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="5">
         <v>1.0197595909860049</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="10">
         <v>-1001119.6713206805</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="5">
         <v>0.95037879495154032</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="10">
         <v>-2709918.1907176636</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="5">
         <v>0.8656809869405927</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="B9" t="s">
+    <row r="9" spans="2:8" ht="12" x14ac:dyDescent="0.2">
+      <c r="B9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="10">
         <v>375541.28358056955</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="5">
         <v>1.0350466917675336</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="10">
         <v>-431127.71733675338</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="5">
         <v>0.95976580769528119</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="10">
         <v>-1425304.4115175437</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="5">
         <v>0.86698611692143168</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="B10" t="s">
+    <row r="10" spans="2:8" ht="12" x14ac:dyDescent="0.2">
+      <c r="B10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="10">
         <v>412197.79724625871</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="5">
         <v>1.0891483469827619</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="10">
         <v>-69556.683930568397</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="5">
         <v>0.98495658289433308</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="10">
         <v>-660687.10493733268</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="5">
         <v>0.85710946620415407</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="B11" t="s">
+    <row r="11" spans="2:8" ht="12" x14ac:dyDescent="0.2">
+      <c r="B11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="10">
         <v>271891.33047977649</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="5">
         <v>1.1402956728729881</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="10">
         <v>4154.1508739702404</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11" s="5">
         <v>1.002143537975452</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="10">
         <v>-270989.0050915496</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="5">
         <v>0.8601699261855339</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="B12" t="s">
+    <row r="12" spans="2:8" ht="12" x14ac:dyDescent="0.2">
+      <c r="B12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="10">
         <v>234768.83116372442</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="5">
         <v>1.0959697692551522</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="10">
         <v>-41154.693742873147</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12" s="5">
         <v>0.98317661487390717</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="10">
         <v>-377107.69700643444</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="5">
         <v>0.84584436321186818</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="B13" t="s">
+    <row r="13" spans="2:8" ht="12" x14ac:dyDescent="0.2">
+      <c r="B13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="10">
         <v>95364.10277619306</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="5">
         <v>1.1198428421942677</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="10">
         <v>-10581.046415620949</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13" s="5">
         <v>0.98670293497319994</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="10">
         <v>-136504.07843101199</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="5">
         <v>0.82845707919389555</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.15">
-      <c r="B14" s="2" t="s">
+    <row r="14" spans="2:8" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="9">
         <v>8174047.6508849859</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="6">
         <v>1.051172768921506</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="11">
         <v>-12011081.501689851</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="6">
         <v>0.92480588266245234</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G14" s="11">
         <v>-35168278.934650123</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="6">
         <v>0.77983267431832548</v>
       </c>
     </row>
+    <row r="15" spans="2:8" ht="11.25" thickTop="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="C2:D2"/>

</xml_diff>